<commit_message>
design changed gh to last edit in menaka
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/malsim khanepaani/valuation malsim khanepaani.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/malsim khanepaani/valuation malsim khanepaani.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A6DE53-57E7-4238-B20B-08EC16B7A709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814476F4-2FE2-4DF8-A736-479CAE56A123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -747,6 +747,75 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -756,75 +825,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1588,89 +1588,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
     </row>
     <row r="2" spans="1:19" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="78" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="A2" s="71" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
     </row>
     <row r="5" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
-      <c r="J5" s="80"/>
-      <c r="K5" s="80"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
     </row>
     <row r="6" spans="1:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="67" t="s">
+      <c r="A6" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
+      <c r="B6" s="74"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
       <c r="G6" s="10"/>
       <c r="H6" s="76" t="s">
         <v>25</v>
@@ -1680,21 +1680,21 @@
       <c r="K6" s="76"/>
     </row>
     <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="84" t="s">
+      <c r="H7" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="84"/>
-      <c r="J7" s="84"/>
-      <c r="K7" s="84"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -2337,11 +2337,11 @@
       <c r="B37" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="81">
+      <c r="C37" s="64">
         <f>J35</f>
         <v>336113.86499999999</v>
       </c>
-      <c r="D37" s="82"/>
+      <c r="D37" s="65"/>
       <c r="E37" s="9">
         <v>100</v>
       </c>
@@ -2363,21 +2363,21 @@
       <c r="B38" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="85">
+      <c r="C38" s="67">
         <v>300000</v>
       </c>
-      <c r="D38" s="86"/>
+      <c r="D38" s="68"/>
       <c r="E38" s="9"/>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B39" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C39" s="85">
+      <c r="C39" s="67">
         <f>C38-C41-C42</f>
         <v>285000</v>
       </c>
-      <c r="D39" s="86"/>
+      <c r="D39" s="68"/>
       <c r="E39" s="9">
         <f>C39/C37*100</f>
         <v>84.79269369027665</v>
@@ -2387,11 +2387,11 @@
       <c r="B40" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C40" s="87">
+      <c r="C40" s="69">
         <f>C37-C39</f>
         <v>51113.864999999991</v>
       </c>
-      <c r="D40" s="87"/>
+      <c r="D40" s="69"/>
       <c r="E40" s="9">
         <f>100-E39</f>
         <v>15.20730630972335</v>
@@ -2401,11 +2401,11 @@
       <c r="B41" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C41" s="81">
+      <c r="C41" s="64">
         <f>C38*0.03</f>
         <v>9000</v>
       </c>
-      <c r="D41" s="82"/>
+      <c r="D41" s="65"/>
       <c r="E41" s="9">
         <v>3</v>
       </c>
@@ -2414,17 +2414,24 @@
       <c r="B42" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C42" s="81">
+      <c r="C42" s="64">
         <f>C38*0.02</f>
         <v>6000</v>
       </c>
-      <c r="D42" s="82"/>
+      <c r="D42" s="65"/>
       <c r="E42" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C41:D41"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="A7:F7"/>
@@ -2433,13 +2440,6 @@
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="C40:D40"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2469,90 +2469,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
     </row>
     <row r="2" spans="1:13" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="71" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
+      <c r="A2" s="80" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
     </row>
     <row r="3" spans="1:13" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="81" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="72"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
-      <c r="I3" s="72"/>
-      <c r="J3" s="72"/>
-      <c r="K3" s="72"/>
+      <c r="B3" s="81"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
     </row>
     <row r="4" spans="1:13" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="72"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="72"/>
-      <c r="H4" s="72"/>
-      <c r="I4" s="72"/>
-      <c r="J4" s="72"/>
-      <c r="K4" s="72"/>
+      <c r="B4" s="81"/>
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
     </row>
     <row r="5" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="82" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="73"/>
-      <c r="D5" s="73"/>
-      <c r="E5" s="73"/>
-      <c r="F5" s="73"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="73"/>
-      <c r="I5" s="73"/>
-      <c r="J5" s="73"/>
-      <c r="K5" s="73"/>
+      <c r="B5" s="82"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="82"/>
+      <c r="H5" s="82"/>
+      <c r="I5" s="82"/>
+      <c r="J5" s="82"/>
+      <c r="K5" s="82"/>
     </row>
     <row r="6" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="45" t="s">
         <v>57</v>
       </c>
       <c r="B6" s="45"/>
-      <c r="C6" s="74">
+      <c r="C6" s="77">
         <f>F27</f>
         <v>336113.86499999999</v>
       </c>
-      <c r="D6" s="75"/>
+      <c r="D6" s="78"/>
       <c r="E6" s="46"/>
       <c r="F6" s="45"/>
       <c r="G6" s="45"/>
@@ -2560,11 +2560,11 @@
         <v>58</v>
       </c>
       <c r="I6" s="45"/>
-      <c r="J6" s="74">
+      <c r="J6" s="77">
         <f>I27</f>
         <v>208459.4124</v>
       </c>
-      <c r="K6" s="75"/>
+      <c r="K6" s="78"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="47" t="s">
@@ -2573,76 +2573,76 @@
       <c r="B7" s="47"/>
       <c r="C7" s="47"/>
       <c r="D7" s="47"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="I7" s="66" t="s">
+      <c r="F7" s="83"/>
+      <c r="G7" s="83"/>
+      <c r="I7" s="84" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="66"/>
-      <c r="K7" s="66"/>
+      <c r="J7" s="84"/>
+      <c r="K7" s="84"/>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="67" t="s">
+      <c r="A8" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="67"/>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="I8" s="68" t="s">
+      <c r="B8" s="74"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="I8" s="85" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="68"/>
-      <c r="K8" s="68"/>
+      <c r="J8" s="85"/>
+      <c r="K8" s="85"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="69" t="str">
+      <c r="A9" s="86" t="str">
         <f>[7]estimate!A7</f>
         <v>Location:- Shankharapur Municipality 1</v>
       </c>
-      <c r="B9" s="69"/>
-      <c r="C9" s="69"/>
-      <c r="D9" s="69"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="I9" s="68" t="s">
+      <c r="B9" s="86"/>
+      <c r="C9" s="86"/>
+      <c r="D9" s="86"/>
+      <c r="E9" s="86"/>
+      <c r="F9" s="86"/>
+      <c r="I9" s="85" t="s">
         <v>71</v>
       </c>
-      <c r="J9" s="68"/>
-      <c r="K9" s="68"/>
+      <c r="J9" s="85"/>
+      <c r="K9" s="85"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="63" t="s">
+      <c r="B11" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="63" t="s">
+      <c r="C11" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="64" t="s">
+      <c r="D11" s="89" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="64"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="64" t="s">
+      <c r="E11" s="89"/>
+      <c r="F11" s="89"/>
+      <c r="G11" s="89" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="64"/>
-      <c r="I11" s="64"/>
-      <c r="J11" s="63" t="s">
+      <c r="H11" s="89"/>
+      <c r="I11" s="89"/>
+      <c r="J11" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="K11" s="62" t="s">
+      <c r="K11" s="87" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="63"/>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
+      <c r="A12" s="88"/>
+      <c r="B12" s="88"/>
+      <c r="C12" s="88"/>
       <c r="D12" s="48" t="s">
         <v>68</v>
       </c>
@@ -2661,8 +2661,8 @@
       <c r="I12" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="63"/>
-      <c r="K12" s="62"/>
+      <c r="J12" s="88"/>
+      <c r="K12" s="87"/>
     </row>
     <row r="13" spans="1:13" s="35" customFormat="1" ht="33" x14ac:dyDescent="0.25">
       <c r="A13" s="49">
@@ -3103,6 +3103,19 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="I9:K9"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -3110,19 +3123,6 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:J12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3155,89 +3155,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="78" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="A2" s="71" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
-      <c r="J5" s="80"/>
-      <c r="K5" s="80"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
     </row>
     <row r="6" spans="1:11" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="67" t="s">
+      <c r="A6" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
+      <c r="B6" s="74"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
       <c r="G6" s="10"/>
       <c r="H6" s="76" t="s">
         <v>25</v>
@@ -3247,21 +3247,21 @@
       <c r="K6" s="76"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="84" t="s">
+      <c r="H7" s="75" t="s">
         <v>70</v>
       </c>
-      <c r="I7" s="84"/>
-      <c r="J7" s="84"/>
-      <c r="K7" s="84"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -4037,11 +4037,11 @@
       <c r="B43" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="81">
+      <c r="C43" s="64">
         <f>J41</f>
         <v>208459.4124</v>
       </c>
-      <c r="D43" s="82"/>
+      <c r="D43" s="65"/>
       <c r="E43" s="9">
         <v>100</v>
       </c>
@@ -4056,21 +4056,21 @@
       <c r="B44" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="85">
+      <c r="C44" s="67">
         <v>300000</v>
       </c>
-      <c r="D44" s="86"/>
+      <c r="D44" s="68"/>
       <c r="E44" s="9"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B45" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C45" s="85">
+      <c r="C45" s="67">
         <f>84.79%*C43</f>
         <v>176752.73577396001</v>
       </c>
-      <c r="D45" s="86"/>
+      <c r="D45" s="68"/>
       <c r="E45" s="9">
         <f>C45/C43*100</f>
         <v>84.79</v>
@@ -4080,11 +4080,11 @@
       <c r="B46" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C46" s="87">
+      <c r="C46" s="69">
         <f>C43-C45</f>
         <v>31706.676626039989</v>
       </c>
-      <c r="D46" s="87"/>
+      <c r="D46" s="69"/>
       <c r="E46" s="9">
         <f>100-E45</f>
         <v>15.209999999999994</v>
@@ -4094,11 +4094,11 @@
       <c r="B47" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C47" s="81">
+      <c r="C47" s="64">
         <f>C44*0.03</f>
         <v>9000</v>
       </c>
-      <c r="D47" s="82"/>
+      <c r="D47" s="65"/>
       <c r="E47" s="9">
         <v>3</v>
       </c>
@@ -4107,24 +4107,17 @@
       <c r="B48" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C48" s="81">
+      <c r="C48" s="64">
         <f>C44*0.02</f>
         <v>6000</v>
       </c>
-      <c r="D48" s="82"/>
+      <c r="D48" s="65"/>
       <c r="E48" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="A7:F7"/>
@@ -4133,6 +4126,13 @@
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
@@ -4162,108 +4162,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="78" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="A2" s="71" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
-      <c r="J5" s="80"/>
-      <c r="K5" s="80"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
     </row>
     <row r="6" spans="1:11" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="67" t="s">
+      <c r="A6" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
+      <c r="B6" s="74"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
       <c r="G6" s="10"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="88"/>
+      <c r="I6" s="63"/>
+      <c r="J6" s="63"/>
       <c r="K6" s="44" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="11"/>
-      <c r="I7" s="89"/>
-      <c r="J7" s="89"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
       <c r="K7" s="43" t="s">
         <v>70</v>
       </c>
@@ -5042,11 +5042,11 @@
       <c r="B43" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="81">
+      <c r="C43" s="64">
         <f>J41</f>
         <v>208459.4124</v>
       </c>
-      <c r="D43" s="82"/>
+      <c r="D43" s="65"/>
       <c r="E43" s="9">
         <v>100</v>
       </c>
@@ -5061,21 +5061,21 @@
       <c r="B44" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="85">
+      <c r="C44" s="67">
         <v>300000</v>
       </c>
-      <c r="D44" s="86"/>
+      <c r="D44" s="68"/>
       <c r="E44" s="9"/>
     </row>
     <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C45" s="85">
+      <c r="C45" s="67">
         <f>84.79%*C43</f>
         <v>176752.73577396001</v>
       </c>
-      <c r="D45" s="86"/>
+      <c r="D45" s="68"/>
       <c r="E45" s="9">
         <f>C45/C43*100</f>
         <v>84.79</v>
@@ -5085,11 +5085,11 @@
       <c r="B46" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C46" s="87">
+      <c r="C46" s="69">
         <f>C43-C45</f>
         <v>31706.676626039989</v>
       </c>
-      <c r="D46" s="87"/>
+      <c r="D46" s="69"/>
       <c r="E46" s="9">
         <f>100-E45</f>
         <v>15.209999999999994</v>
@@ -5099,11 +5099,11 @@
       <c r="B47" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C47" s="81">
+      <c r="C47" s="64">
         <f>C44*0.03</f>
         <v>9000</v>
       </c>
-      <c r="D47" s="82"/>
+      <c r="D47" s="65"/>
       <c r="E47" s="9">
         <v>3</v>
       </c>
@@ -5112,17 +5112,23 @@
       <c r="B48" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C48" s="81">
+      <c r="C48" s="64">
         <f>C44*0.02</f>
         <v>6000</v>
       </c>
-      <c r="D48" s="82"/>
+      <c r="D48" s="65"/>
       <c r="E48" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="A7:F7"/>
@@ -5130,12 +5136,6 @@
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="95" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -5166,89 +5166,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
     </row>
     <row r="2" spans="1:19" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="78" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="A2" s="71" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
+      <c r="K3" s="72"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
     </row>
     <row r="5" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
-      <c r="J5" s="80"/>
-      <c r="K5" s="80"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
     </row>
     <row r="6" spans="1:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="67" t="s">
+      <c r="A6" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
+      <c r="B6" s="74"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
       <c r="G6" s="10"/>
       <c r="H6" s="76" t="s">
         <v>25</v>
@@ -5258,21 +5258,21 @@
       <c r="K6" s="76"/>
     </row>
     <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="84" t="s">
+      <c r="H7" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="84"/>
-      <c r="J7" s="84"/>
-      <c r="K7" s="84"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -5897,11 +5897,11 @@
       <c r="B36" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="81">
+      <c r="C36" s="64">
         <f>J34</f>
         <v>335761.30499999999</v>
       </c>
-      <c r="D36" s="82"/>
+      <c r="D36" s="65"/>
       <c r="E36" s="9">
         <v>100</v>
       </c>
@@ -5923,21 +5923,21 @@
       <c r="B37" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="85">
+      <c r="C37" s="67">
         <v>300000</v>
       </c>
-      <c r="D37" s="86"/>
+      <c r="D37" s="68"/>
       <c r="E37" s="9"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B38" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C38" s="85">
+      <c r="C38" s="67">
         <f>C37-C40-C41</f>
         <v>285000</v>
       </c>
-      <c r="D38" s="86"/>
+      <c r="D38" s="68"/>
       <c r="E38" s="9">
         <f>C38/C36*100</f>
         <v>84.881728703073762</v>
@@ -5947,11 +5947,11 @@
       <c r="B39" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C39" s="87">
+      <c r="C39" s="69">
         <f>C36-C38</f>
         <v>50761.304999999993</v>
       </c>
-      <c r="D39" s="87"/>
+      <c r="D39" s="69"/>
       <c r="E39" s="9">
         <f>100-E38</f>
         <v>15.118271296926238</v>
@@ -5961,11 +5961,11 @@
       <c r="B40" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C40" s="81">
+      <c r="C40" s="64">
         <f>C37*0.03</f>
         <v>9000</v>
       </c>
-      <c r="D40" s="82"/>
+      <c r="D40" s="65"/>
       <c r="E40" s="9">
         <v>3</v>
       </c>
@@ -5974,24 +5974,17 @@
       <c r="B41" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C41" s="81">
+      <c r="C41" s="64">
         <f>C37*0.02</f>
         <v>6000</v>
       </c>
-      <c r="D41" s="82"/>
+      <c r="D41" s="65"/>
       <c r="E41" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C41:D41"/>
     <mergeCell ref="A7:F7"/>
@@ -6000,6 +5993,13 @@
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C39:D39"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>